<commit_message>
Add 5-year projection tab to financial model
Census ramp, debt amortization schedule, taxes, free cash flow to
equity, and equity IRR/MOIC with a Year-5 exit. New projection
assumptions added to the Assumptions tab.

https://claude.ai/code/session_01KCj9t7yChzrUxrNjnU9Cnv
</commit_message>
<xml_diff>
--- a/staffing-agency-plan/Staffing_Agency_Financial_Model.xlsx
+++ b/staffing-agency-plan/Staffing_Agency_Financial_Model.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Unit Economics" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Working Capital" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Acquisition" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="5-Year Projection" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,12 +21,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0&quot;x&quot;"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="$#,##0"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="169" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -112,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -136,6 +138,8 @@
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -501,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="102" customWidth="1" min="1" max="1"/>
@@ -584,62 +588,69 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5. 5-Year Projection - census ramp, debt amortization, taxes, FCFE, and equity IRR/MOIC.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>GROUNDING (Texas / San Antonio, 2025-2026 - verify before relying)</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - TX Medicaid attendant rates support avg ~$13.00/hr wage + 14-15% payroll-tax/benefits (Sept 2025).</t>
+          <t>GROUNDING (Texas / San Antonio, 2025-2026 - verify before relying)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - On Medicaid work, margin comes from overhead efficiency &amp; scale, NOT rate negotiation (capped).</t>
+          <t xml:space="preserve">  - TX Medicaid attendant rates support avg ~$13.00/hr wage + 14-15% payroll-tax/benefits (Sept 2025).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Staffing markup typically 1.45x-1.75x of pay; gross margin ~15-30%.</t>
+          <t xml:space="preserve">  - On Medicaid work, margin comes from overhead efficiency &amp; scale, NOT rate negotiation (capped).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Payroll float: pay DSPs weekly, collect from Medicaid/MCOs in 30-90 days. Fund it or factor.</t>
+          <t xml:space="preserve">  - Staffing markup typically 1.45x-1.75x of pay; gross margin ~15-30%.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Small agencies ($0.5-3M rev) trade ~2-3.5x SDE; IDD/HCS ~4-7x EBITDA (small), 8-11x (platform).</t>
+          <t xml:space="preserve">  - Payroll float: pay DSPs weekly, collect from Medicaid/MCOs in 30-90 days. Fund it or factor.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t xml:space="preserve">  - Small agencies ($0.5-3M rev) trade ~2-3.5x SDE; IDD/HCS ~4-7x EBITDA (small), 8-11x (platform).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - Caregiver turnover median ~75% (2024) - the #1 operational risk.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-    </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>These are starting assumptions, not guarantees. Replace with real diligence numbers.</t>
         </is>
@@ -656,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1102,6 +1113,105 @@
       <c r="C37" s="9" t="inlineStr">
         <is>
           <t>What you raise from investors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>5-YEAR PROJECTION</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="n"/>
+      <c r="C39" s="7" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Annual revenue growth (census ramp) %</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Organic census growth/yr. Slot freeze caps HCS upside - be realistic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>EBITDA margin improvement (pp/yr)</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>Scale efficiency. 0.005 = +0.5 point/yr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Annual D&amp;A (goodwill/intangible amort.)</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="n">
+        <v>75000</v>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Asset-deal intangibles amortize ~15yr (Sec.197). ~price/15.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Effective tax rate %</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>Use ~21% C-corp; set 0 if pass-through taxed at owner level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Debt amortization term (years)</t>
+        </is>
+      </c>
+      <c r="B44" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>e.g., SBA 7(a) ~10yr; seller note shorter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Exit multiple (x Yr-5 EBITDA)</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Terminal value at sale. Scale earns a higher multiple.</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1278,7 @@
         </is>
       </c>
       <c r="B5" s="14">
-        <f>'Assumptions'!B4*('Assumptions'!B11+'Assumptions'!B12+'Assumptions'!B13)</f>
+        <f>'Assumptions'!B4*('Assumptions'!B43+'Assumptions'!B12+'Assumptions'!B13)</f>
         <v/>
       </c>
     </row>
@@ -1701,4 +1811,621 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>5-Year Projection &amp; Equity Returns</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="n"/>
+      <c r="C1" s="3" t="n"/>
+      <c r="D1" s="3" t="n"/>
+      <c r="E1" s="3" t="n"/>
+      <c r="F1" s="3" t="n"/>
+      <c r="G1" s="3" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>(all figures by operating year)</t>
+        </is>
+      </c>
+      <c r="B2" s="23" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="C2" s="23" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="D2" s="23" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="E2" s="23" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="F2" s="23" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>OPERATING PROJECTION</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="7" t="n"/>
+      <c r="F3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B4" s="18">
+        <f>'Acquisition'!B3*(1+'Assumptions'!B40)</f>
+        <v/>
+      </c>
+      <c r="C4" s="18">
+        <f>B4*(1+'Assumptions'!B40)</f>
+        <v/>
+      </c>
+      <c r="D4" s="18">
+        <f>C4*(1+'Assumptions'!B40)</f>
+        <v/>
+      </c>
+      <c r="E4" s="18">
+        <f>D4*(1+'Assumptions'!B40)</f>
+        <v/>
+      </c>
+      <c r="F4" s="18">
+        <f>E4*(1+'Assumptions'!B40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EBITDA margin %</t>
+        </is>
+      </c>
+      <c r="B5" s="16">
+        <f>'Acquisition'!B4+'Assumptions'!B41*1</f>
+        <v/>
+      </c>
+      <c r="C5" s="16">
+        <f>'Acquisition'!B4+'Assumptions'!B41*2</f>
+        <v/>
+      </c>
+      <c r="D5" s="16">
+        <f>'Acquisition'!B4+'Assumptions'!B41*3</f>
+        <v/>
+      </c>
+      <c r="E5" s="16">
+        <f>'Acquisition'!B4+'Assumptions'!B41*4</f>
+        <v/>
+      </c>
+      <c r="F5" s="16">
+        <f>'Acquisition'!B4+'Assumptions'!B41*5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B6" s="18">
+        <f>B4*B5</f>
+        <v/>
+      </c>
+      <c r="C6" s="18">
+        <f>C4*C5</f>
+        <v/>
+      </c>
+      <c r="D6" s="18">
+        <f>D4*D5</f>
+        <v/>
+      </c>
+      <c r="E6" s="18">
+        <f>E4*E5</f>
+        <v/>
+      </c>
+      <c r="F6" s="18">
+        <f>F4*F5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Less: D&amp;A</t>
+        </is>
+      </c>
+      <c r="B7" s="19">
+        <f>-'Assumptions'!B42</f>
+        <v/>
+      </c>
+      <c r="C7" s="19">
+        <f>-'Assumptions'!B42</f>
+        <v/>
+      </c>
+      <c r="D7" s="19">
+        <f>-'Assumptions'!B42</f>
+        <v/>
+      </c>
+      <c r="E7" s="19">
+        <f>-'Assumptions'!B42</f>
+        <v/>
+      </c>
+      <c r="F7" s="19">
+        <f>-'Assumptions'!B42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>EBIT</t>
+        </is>
+      </c>
+      <c r="B8" s="19">
+        <f>B6+B7</f>
+        <v/>
+      </c>
+      <c r="C8" s="19">
+        <f>C6+C7</f>
+        <v/>
+      </c>
+      <c r="D8" s="19">
+        <f>D6+D7</f>
+        <v/>
+      </c>
+      <c r="E8" s="19">
+        <f>E6+E7</f>
+        <v/>
+      </c>
+      <c r="F8" s="19">
+        <f>F6+F7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>DEBT SCHEDULE</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Beginning debt balance</t>
+        </is>
+      </c>
+      <c r="B10" s="19">
+        <f>'Acquisition'!B12</f>
+        <v/>
+      </c>
+      <c r="C10" s="19">
+        <f>B14</f>
+        <v/>
+      </c>
+      <c r="D10" s="19">
+        <f>C14</f>
+        <v/>
+      </c>
+      <c r="E10" s="19">
+        <f>D14</f>
+        <v/>
+      </c>
+      <c r="F10" s="19">
+        <f>E14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Annual debt payment (P&amp;I)</t>
+        </is>
+      </c>
+      <c r="B11" s="19">
+        <f>IF(B10&gt;0,MIN(-PMT('Assumptions'!B36,'Assumptions'!B44,'Acquisition'!B12),B10+B10*'Assumptions'!B36),0)</f>
+        <v/>
+      </c>
+      <c r="C11" s="19">
+        <f>IF(C10&gt;0,MIN(-PMT('Assumptions'!B36,'Assumptions'!B44,'Acquisition'!B12),C10+C10*'Assumptions'!B36),0)</f>
+        <v/>
+      </c>
+      <c r="D11" s="19">
+        <f>IF(D10&gt;0,MIN(-PMT('Assumptions'!B36,'Assumptions'!B44,'Acquisition'!B12),D10+D10*'Assumptions'!B36),0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="19">
+        <f>IF(E10&gt;0,MIN(-PMT('Assumptions'!B36,'Assumptions'!B44,'Acquisition'!B12),E10+E10*'Assumptions'!B36),0)</f>
+        <v/>
+      </c>
+      <c r="F11" s="19">
+        <f>IF(F10&gt;0,MIN(-PMT('Assumptions'!B36,'Assumptions'!B44,'Acquisition'!B12),F10+F10*'Assumptions'!B36),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Interest</t>
+        </is>
+      </c>
+      <c r="B12" s="19">
+        <f>B10*'Assumptions'!B36</f>
+        <v/>
+      </c>
+      <c r="C12" s="19">
+        <f>C10*'Assumptions'!B36</f>
+        <v/>
+      </c>
+      <c r="D12" s="19">
+        <f>D10*'Assumptions'!B36</f>
+        <v/>
+      </c>
+      <c r="E12" s="19">
+        <f>E10*'Assumptions'!B36</f>
+        <v/>
+      </c>
+      <c r="F12" s="19">
+        <f>F10*'Assumptions'!B36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Principal</t>
+        </is>
+      </c>
+      <c r="B13" s="19">
+        <f>B11-B12</f>
+        <v/>
+      </c>
+      <c r="C13" s="19">
+        <f>C11-C12</f>
+        <v/>
+      </c>
+      <c r="D13" s="19">
+        <f>D11-D12</f>
+        <v/>
+      </c>
+      <c r="E13" s="19">
+        <f>E11-E12</f>
+        <v/>
+      </c>
+      <c r="F13" s="19">
+        <f>F11-F12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ending debt balance</t>
+        </is>
+      </c>
+      <c r="B14" s="19">
+        <f>MAX(0,B10-B13)</f>
+        <v/>
+      </c>
+      <c r="C14" s="19">
+        <f>MAX(0,C10-C13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="19">
+        <f>MAX(0,D10-D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="19">
+        <f>MAX(0,E10-E13)</f>
+        <v/>
+      </c>
+      <c r="F14" s="19">
+        <f>MAX(0,F10-F13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>TAXES &amp; NET INCOME</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Pre-tax income (EBIT - interest)</t>
+        </is>
+      </c>
+      <c r="B16" s="19">
+        <f>B8-B12</f>
+        <v/>
+      </c>
+      <c r="C16" s="19">
+        <f>C8-C12</f>
+        <v/>
+      </c>
+      <c r="D16" s="19">
+        <f>D8-D12</f>
+        <v/>
+      </c>
+      <c r="E16" s="19">
+        <f>E8-E12</f>
+        <v/>
+      </c>
+      <c r="F16" s="19">
+        <f>F8-F12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Less: taxes</t>
+        </is>
+      </c>
+      <c r="B17" s="19">
+        <f>-MAX(0,B16*'Assumptions'!B43)</f>
+        <v/>
+      </c>
+      <c r="C17" s="19">
+        <f>-MAX(0,C16*'Assumptions'!B43)</f>
+        <v/>
+      </c>
+      <c r="D17" s="19">
+        <f>-MAX(0,D16*'Assumptions'!B43)</f>
+        <v/>
+      </c>
+      <c r="E17" s="19">
+        <f>-MAX(0,E16*'Assumptions'!B43)</f>
+        <v/>
+      </c>
+      <c r="F17" s="19">
+        <f>-MAX(0,F16*'Assumptions'!B43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Net income</t>
+        </is>
+      </c>
+      <c r="B18" s="18">
+        <f>B16+B17</f>
+        <v/>
+      </c>
+      <c r="C18" s="18">
+        <f>C16+C17</f>
+        <v/>
+      </c>
+      <c r="D18" s="18">
+        <f>D16+D17</f>
+        <v/>
+      </c>
+      <c r="E18" s="18">
+        <f>E16+E17</f>
+        <v/>
+      </c>
+      <c r="F18" s="18">
+        <f>F16+F17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>FREE CASH FLOW TO EQUITY</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>FCFE (NI + D&amp;A - principal)</t>
+        </is>
+      </c>
+      <c r="B20" s="18">
+        <f>B18-B7-B13</f>
+        <v/>
+      </c>
+      <c r="C20" s="18">
+        <f>C18-C7-C13</f>
+        <v/>
+      </c>
+      <c r="D20" s="18">
+        <f>D18-D7-D13</f>
+        <v/>
+      </c>
+      <c r="E20" s="18">
+        <f>E18-E7-E13</f>
+        <v/>
+      </c>
+      <c r="F20" s="18">
+        <f>F18-F7-F13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>EQUITY RETURNS</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr"/>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>Year 0</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="D23" s="23" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="E23" s="23" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="F23" s="23" t="inlineStr">
+        <is>
+          <t>Year 4</t>
+        </is>
+      </c>
+      <c r="G23" s="23" t="inlineStr">
+        <is>
+          <t>Year 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Terminal equity value (Yr5 sale)</t>
+        </is>
+      </c>
+      <c r="G24" s="18">
+        <f>F6*'Assumptions'!B45-F14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Equity cash flow</t>
+        </is>
+      </c>
+      <c r="B25" s="18">
+        <f>-'Acquisition'!B13</f>
+        <v/>
+      </c>
+      <c r="C25" s="18">
+        <f>B20</f>
+        <v/>
+      </c>
+      <c r="D25" s="18">
+        <f>C20</f>
+        <v/>
+      </c>
+      <c r="E25" s="18">
+        <f>D20</f>
+        <v/>
+      </c>
+      <c r="F25" s="18">
+        <f>E20</f>
+        <v/>
+      </c>
+      <c r="G25" s="18">
+        <f>F20+G24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Equity IRR (5-yr)</t>
+        </is>
+      </c>
+      <c r="B27" s="21">
+        <f>IRR(B25:G25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Equity MOIC (5-yr)</t>
+        </is>
+      </c>
+      <c r="B28" s="24">
+        <f>SUM(C25:G25)/-B25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Assumes: organic census growth, constant exit multiple, interest-only-then-amortizing debt per term,</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>and a Year-5 sale at the exit multiple. Stress-test growth &amp; exit multiple - HCS slot freeze caps upside.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>